<commit_message>
[tools] Excel evaluation: fold LibreOffice's respellings when comparing styles; explicit fonts in the inputs
</commit_message>
<xml_diff>
--- a/office-agent/evals/xlsx/tasks/05-edit-budget/inputs/budget_q1.xlsx
+++ b/office-agent/evals/xlsx/tasks/05-edit-budget/inputs/budget_q1.xlsx
@@ -28,11 +28,15 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <i val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">

</xml_diff>